<commit_message>
fix: issue with validation resolved
</commit_message>
<xml_diff>
--- a/LAMP-DTR-Tracker.xlsx
+++ b/LAMP-DTR-Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\justi\Documents\UiPath\AppDevt Finals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B61F123-8645-499E-8AF4-ACABA0695CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC5F895-3666-46E7-96F5-E2E3C5D05838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="3" xr2:uid="{4768BDF5-CECC-48E1-A5D4-20995DBA131C}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="28">
   <si>
     <t>Student ID</t>
   </si>
@@ -123,6 +123,9 @@
   </si>
   <si>
     <t>justinnnerip+jose@gmail.com</t>
+  </si>
+  <si>
+    <t>September 2026</t>
   </si>
 </sst>
 </file>
@@ -184,18 +187,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -204,9 +201,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -621,12 +625,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AAC47F8-9D20-45AE-992C-C05395EFFC25}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.1328125" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.46484375" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="27.75" x14ac:dyDescent="0.45">
@@ -644,10 +648,10 @@
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3">
-        <v>46266</v>
-      </c>
-      <c r="C2" s="4">
+      <c r="B2" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="9">
         <v>46302</v>
       </c>
     </row>
@@ -655,12 +659,108 @@
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3">
-        <v>46266</v>
-      </c>
-      <c r="C3" s="4">
+      <c r="B3" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="9">
         <v>46311</v>
       </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -680,28 +780,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.75" x14ac:dyDescent="0.45">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="3" t="s">
         <v>16</v>
       </c>
     </row>
@@ -715,16 +815,16 @@
       <c r="C2" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="7">
-        <v>46266</v>
+      <c r="D2" s="10">
+        <v>46296</v>
       </c>
       <c r="F2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="6">
+      <c r="I2">
         <v>0</v>
       </c>
     </row>
@@ -738,16 +838,16 @@
       <c r="C3" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="7">
-        <v>46266</v>
+      <c r="D3" s="10">
+        <v>46296</v>
       </c>
       <c r="F3" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3">
         <v>0</v>
       </c>
     </row>
@@ -761,16 +861,16 @@
       <c r="C4" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="7">
-        <v>46266</v>
+      <c r="D4" s="10">
+        <v>46296</v>
       </c>
       <c r="F4" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4">
         <v>5</v>
       </c>
     </row>
@@ -784,8 +884,8 @@
       <c r="C5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="7">
-        <v>46266</v>
+      <c r="D5" s="10">
+        <v>46296</v>
       </c>
       <c r="F5" t="s">
         <v>19</v>
@@ -798,8 +898,8 @@
       <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="7">
-        <v>46266</v>
+      <c r="D6" s="10">
+        <v>46296</v>
       </c>
       <c r="F6" t="s">
         <v>19</v>
@@ -812,7 +912,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2B44BF7-DFFC-4E9D-804A-16394639C373}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="14.3984375" customWidth="1"/>
@@ -821,22 +921,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" x14ac:dyDescent="0.45">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="3" t="s">
         <v>21</v>
       </c>
     </row>
@@ -850,10 +950,10 @@
       <c r="C2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="5">
         <v>46291</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="6">
         <v>46310</v>
       </c>
       <c r="F2" t="s">
@@ -862,19 +962,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" s="8">
+        <v>26</v>
+      </c>
+      <c r="D3" s="5">
         <v>46291</v>
       </c>
-      <c r="E3" s="9">
-        <v>46324</v>
+      <c r="E3" s="6">
+        <v>46325</v>
       </c>
       <c r="F3" t="s">
         <v>22</v>
@@ -882,301 +982,21 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="8">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5">
         <v>46291</v>
       </c>
-      <c r="E4" s="9">
-        <v>46324</v>
+      <c r="E4" s="6">
+        <v>46325</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="8">
-        <v>46291</v>
-      </c>
-      <c r="E5" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="8">
-        <v>46291</v>
-      </c>
-      <c r="E6" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="8">
-        <v>46291</v>
-      </c>
-      <c r="E7" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="8">
-        <v>46291</v>
-      </c>
-      <c r="E8" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="8">
-        <v>46291</v>
-      </c>
-      <c r="E9" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="8">
-        <v>46291</v>
-      </c>
-      <c r="E10" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="8">
-        <v>46321</v>
-      </c>
-      <c r="E11" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="8">
-        <v>46321</v>
-      </c>
-      <c r="E12" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" t="s">
-        <v>26</v>
-      </c>
-      <c r="D13" s="8">
-        <v>46321</v>
-      </c>
-      <c r="E13" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F13" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="8">
-        <v>46321</v>
-      </c>
-      <c r="E14" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F14" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="7">
-        <v>46266</v>
-      </c>
-      <c r="E15" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F15" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" t="s">
-        <v>25</v>
-      </c>
-      <c r="D16" s="7">
-        <v>46266</v>
-      </c>
-      <c r="E16" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" t="s">
-        <v>26</v>
-      </c>
-      <c r="D17" s="7">
-        <v>46266</v>
-      </c>
-      <c r="E17" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F17" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="7">
-        <v>46266</v>
-      </c>
-      <c r="E18" s="9">
-        <v>46324</v>
-      </c>
-      <c r="F18" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(logs): fixed incorrect results in logs and improved validation
</commit_message>
<xml_diff>
--- a/LAMP-DTR-Tracker.xlsx
+++ b/LAMP-DTR-Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\justi\Documents\UiPath\AppDevt Finals\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dlsleduph-my.sharepoint.com/personal/marielle_anne_collera_dlsl_edu_ph/Documents/School/A.Y. 2026-2027/Appdevt/appdevt-finals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC5F895-3666-46E7-96F5-E2E3C5D05838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{ADC5F895-3666-46E7-96F5-E2E3C5D05838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{749DE749-C120-474E-ACAC-34FF42A3AFB4}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="3" xr2:uid="{4768BDF5-CECC-48E1-A5D4-20995DBA131C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="3" xr2:uid="{4768BDF5-CECC-48E1-A5D4-20995DBA131C}"/>
   </bookViews>
   <sheets>
     <sheet name="Roster" sheetId="1" r:id="rId1"/>
@@ -226,6 +226,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -546,14 +550,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86290173-4BB9-4CA0-AC7C-5D9A2752C291}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.3984375" customWidth="1"/>
-    <col min="2" max="2" width="19.86328125" customWidth="1"/>
-    <col min="3" max="3" width="24.33203125" customWidth="1"/>
+    <col min="1" max="1" width="12.36328125" customWidth="1"/>
+    <col min="2" max="2" width="19.81640625" customWidth="1"/>
+    <col min="3" max="3" width="24.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -564,7 +568,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="27" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -575,7 +579,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="27" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -586,7 +590,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="27" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -597,7 +601,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="27" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -608,7 +612,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
@@ -626,14 +630,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AAC47F8-9D20-45AE-992C-C05395EFFC25}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.46484375" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" customWidth="1"/>
+    <col min="3" max="3" width="11.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -644,7 +648,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -655,7 +659,7 @@
         <v>46302</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" ht="28" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -666,99 +670,99 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
     </row>
@@ -770,16 +774,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67935AA9-FD21-482D-9CFF-DFADA775544C}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="9.33203125" customWidth="1"/>
+    <col min="1" max="3" width="9.36328125" customWidth="1"/>
     <col min="4" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.3984375" customWidth="1"/>
-    <col min="9" max="9" width="6.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.36328125" customWidth="1"/>
+    <col min="9" max="9" width="6.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -805,7 +809,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -828,7 +832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="27" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:9" ht="28" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -851,7 +855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -874,7 +878,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -891,7 +895,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -913,14 +917,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2B44BF7-DFFC-4E9D-804A-16394639C373}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="14.3984375" customWidth="1"/>
-    <col min="3" max="3" width="27.86328125" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="14.36328125" customWidth="1"/>
+    <col min="3" max="3" width="27.81640625" customWidth="1"/>
+    <col min="4" max="4" width="13.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="27.75" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -940,7 +944,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -960,7 +964,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -980,7 +984,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1006,6 +1010,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010093AF9BF61107EB45B8924CB8347B1520" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="83f8879dc2bdd2115b7d8e7635e8ea05">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="e086d1b4-0fa7-4576-91a3-91f0e571aacc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac0cef59c1f934e89cb01f30ccaa858e" ns3:_="">
     <xsd:import namespace="e086d1b4-0fa7-4576-91a3-91f0e571aacc"/>
@@ -1155,22 +1174,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3950F8B8-4E67-4023-AD00-ACA89CC7C775}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="e086d1b4-0fa7-4576-91a3-91f0e571aacc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19927099-1B40-4023-A667-F2B28A775791}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA3B881A-04C5-49E6-ACC8-D853EBF11F77}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1186,28 +1214,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19927099-1B40-4023-A667-F2B28A775791}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3950F8B8-4E67-4023-AD00-ACA89CC7C775}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="e086d1b4-0fa7-4576-91a3-91f0e571aacc"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>